<commit_message>
Update leave data - 2026-07-17T09:35:11.293Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,10 +400,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:D2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Employee ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Department</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Date of Joining</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EMP001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Anil Kumar Sharma</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -430,10 +459,45 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Employee ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Earned Leave Quota</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Leave Taken</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Leave Balance</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EMP001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Anil Kumar Sharma</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:38:27.194Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,9 +430,23 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Support Staff</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -459,7 +473,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -495,9 +509,26 @@
         <v>20</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:41:05.471Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,9 +444,23 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EMP003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Devesh Jaju</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -473,7 +487,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -526,9 +540,26 @@
         <v>20</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EMP003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Devesh Jaju</v>
+      </c>
+      <c r="C4">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:42:38.595Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -458,9 +458,37 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EMP004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Kushal Vagela</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Sales Support</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>EMP005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mahesh Sharma</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Production</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -487,7 +515,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -557,9 +585,43 @@
         <v>20</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EMP004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Kushal Vagela</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>EMP005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mahesh Sharma</v>
+      </c>
+      <c r="C6">
+        <v>20</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:45:10.415Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -486,9 +486,37 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>EMP006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Om Prakesh</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Sales and Support</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>EMP007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Vikash Sharma</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ERP Support</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -515,7 +543,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -619,9 +647,43 @@
         <v>20</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>EMP006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Om Prakesh</v>
+      </c>
+      <c r="C7">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>EMP007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Vikash Sharma</v>
+      </c>
+      <c r="C8">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:46:46.865Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -514,9 +514,23 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Vinod</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Vishwakarma</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Account</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -543,7 +557,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -681,9 +695,26 @@
         <v>20</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Vinod</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Vishwakarma</v>
+      </c>
+      <c r="C9">
+        <v>20</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:48:48.268Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -516,10 +516,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Vinod</v>
+        <v>EMP008</v>
       </c>
       <c r="B9" t="str">
-        <v>Vishwakarma</v>
+        <v>Vinod Vishwakarma</v>
       </c>
       <c r="C9" t="str">
         <v>Account</v>
@@ -528,9 +528,23 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>EMP009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Akash</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Account</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -557,7 +571,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -697,10 +711,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Vinod</v>
+        <v>EMP008</v>
       </c>
       <c r="B9" t="str">
-        <v>Vishwakarma</v>
+        <v>Vinod Vishwakarma</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -709,12 +723,29 @@
         <v>0</v>
       </c>
       <c r="E9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>EMP009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Akash</v>
+      </c>
+      <c r="C10">
+        <v>20</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:50:10.044Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -536,15 +536,29 @@
         <v>Akash</v>
       </c>
       <c r="C10" t="str">
-        <v>Account</v>
+        <v>Support Staff</v>
       </c>
       <c r="D10" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>EMP010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ashok</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Support Staff</v>
+      </c>
+      <c r="D11" t="str">
         <v>2026-07-01</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -571,7 +585,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -743,9 +757,26 @@
         <v>20</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>EMP010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ashok</v>
+      </c>
+      <c r="C11">
+        <v>20</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:51:24.434Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -556,9 +556,37 @@
         <v>2026-07-01</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>EMP011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Dipaknath Jogi</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Support Staff</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>EMP012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Praveen</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Tata</v>
+      </c>
+      <c r="D13" t="str">
+        <v>2026-07-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -585,7 +613,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -774,9 +802,43 @@
         <v>20</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>EMP011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Dipaknath Jogi</v>
+      </c>
+      <c r="C12">
+        <v>20</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>EMP012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Praveen</v>
+      </c>
+      <c r="C13">
+        <v>20</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-07-17T09:52:48.133Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -550,7 +550,7 @@
         <v>Ashok</v>
       </c>
       <c r="C11" t="str">
-        <v>Support Staff</v>
+        <v>Tata</v>
       </c>
       <c r="D11" t="str">
         <v>2026-07-01</v>
@@ -593,10 +593,80 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Employee ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>From</v>
+      </c>
+      <c r="D1" t="str">
+        <v>To</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Days</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Reason</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Sick</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -660,10 +730,10 @@
         <v>20</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -762,10 +832,10 @@
         <v>20</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Update leave data - 2026-08-01T13:30:37.435Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -6,7 +6,8 @@
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
     <sheet name="Leave Records" sheetId="2" r:id="rId2"/>
     <sheet name="Public Holidays" sheetId="3" r:id="rId3"/>
-    <sheet name="Leave Balance" sheetId="4" r:id="rId4"/>
+    <sheet name="Comp Off Credits" sheetId="4" r:id="rId4"/>
+    <sheet name="Leave Balance" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -683,7 +684,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -696,10 +707,28 @@
         <v>Earned Leave Quota</v>
       </c>
       <c r="D1" t="str">
-        <v>Leave Taken</v>
+        <v>Earned Leave Taken</v>
       </c>
       <c r="E1" t="str">
-        <v>Leave Balance</v>
+        <v>Earned Leave Balance</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Sick Leave Quota</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Sick Leave Taken</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Sick Leave Balance</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Comp Off Credited</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Comp Off Taken</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Comp Off Balance</v>
       </c>
     </row>
     <row r="2">
@@ -718,6 +747,24 @@
       <c r="E2">
         <v>20</v>
       </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -735,6 +782,24 @@
       <c r="E3">
         <v>19</v>
       </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>10</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -752,6 +817,24 @@
       <c r="E4">
         <v>20</v>
       </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -769,6 +852,24 @@
       <c r="E5">
         <v>20</v>
       </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -786,6 +887,24 @@
       <c r="E6">
         <v>20</v>
       </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -803,6 +922,24 @@
       <c r="E7">
         <v>20</v>
       </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -820,6 +957,24 @@
       <c r="E8">
         <v>20</v>
       </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -837,6 +992,24 @@
       <c r="E9">
         <v>19</v>
       </c>
+      <c r="F9">
+        <v>10</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -854,6 +1027,24 @@
       <c r="E10">
         <v>20</v>
       </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>10</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -871,6 +1062,24 @@
       <c r="E11">
         <v>20</v>
       </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>10</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -888,6 +1097,24 @@
       <c r="E12">
         <v>20</v>
       </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>10</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -905,10 +1132,28 @@
       <c r="E13">
         <v>20</v>
       </c>
+      <c r="F13">
+        <v>10</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>10</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update leave data - 2026-08-01T13:33:34.735Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,39 +621,39 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B2" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E2" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP008</v>
+        <v>EMP002</v>
       </c>
       <c r="B3" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Arvind</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="E3" t="str">
         <v>Earned</v>
@@ -662,12 +662,35 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -739,13 +762,13 @@
         <v>Anil Kumar Sharma</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -774,13 +797,13 @@
         <v>Arvind</v>
       </c>
       <c r="C3">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F3">
         <v>10</v>
@@ -809,13 +832,13 @@
         <v>Devesh Jaju</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F4">
         <v>10</v>
@@ -844,13 +867,13 @@
         <v>Kushal Vagela</v>
       </c>
       <c r="C5">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F5">
         <v>10</v>
@@ -879,13 +902,13 @@
         <v>Mahesh Sharma</v>
       </c>
       <c r="C6">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F6">
         <v>10</v>
@@ -914,13 +937,13 @@
         <v>Om Prakesh</v>
       </c>
       <c r="C7">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F7">
         <v>10</v>
@@ -949,13 +972,13 @@
         <v>Vikash Sharma</v>
       </c>
       <c r="C8">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F8">
         <v>10</v>
@@ -984,13 +1007,13 @@
         <v>Vinod Vishwakarma</v>
       </c>
       <c r="C9">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F9">
         <v>10</v>
@@ -1019,22 +1042,22 @@
         <v>Akash</v>
       </c>
       <c r="C10">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F10">
         <v>10</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1054,13 +1077,13 @@
         <v>Ashok</v>
       </c>
       <c r="C11">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F11">
         <v>10</v>
@@ -1089,13 +1112,13 @@
         <v>Dipaknath Jogi</v>
       </c>
       <c r="C12">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F12">
         <v>10</v>
@@ -1124,13 +1147,13 @@
         <v>Praveen</v>
       </c>
       <c r="C13">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F13">
         <v>10</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-03T07:09:51.131Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -679,7 +679,7 @@
         <v>2026-07-14</v>
       </c>
       <c r="E4" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -771,13 +771,13 @@
         <v>12</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -806,13 +806,13 @@
         <v>11</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -841,13 +841,13 @@
         <v>12</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -876,13 +876,13 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -911,13 +911,13 @@
         <v>12</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -946,13 +946,13 @@
         <v>12</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -981,13 +981,13 @@
         <v>12</v>
       </c>
       <c r="F8">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -1010,19 +1010,19 @@
         <v>12</v>
       </c>
       <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>12</v>
+      </c>
+      <c r="F9">
+        <v>5</v>
+      </c>
+      <c r="G9">
         <v>1</v>
       </c>
-      <c r="E9">
-        <v>11</v>
-      </c>
-      <c r="F9">
-        <v>10</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
       <c r="H9">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1051,13 +1051,13 @@
         <v>12</v>
       </c>
       <c r="F10">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
       <c r="H10">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1086,13 +1086,13 @@
         <v>12</v>
       </c>
       <c r="F11">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -1121,13 +1121,13 @@
         <v>12</v>
       </c>
       <c r="F12">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -1156,13 +1156,13 @@
         <v>12</v>
       </c>
       <c r="F13">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I13">
         <v>0</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-12T06:17:20.644Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,16 +621,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP009</v>
+        <v>EMP002</v>
       </c>
       <c r="B2" t="str">
-        <v>Akash</v>
+        <v>Arvind</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E2" t="str">
         <v>Sick</v>
@@ -644,39 +644,39 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP002</v>
+        <v>EMP001</v>
       </c>
       <c r="B3" t="str">
-        <v>Arvind</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-07-16</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-07-16</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E3" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP008</v>
+        <v>EMP009</v>
       </c>
       <c r="B4" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Akash</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-07-14</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-07-14</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E4" t="str">
         <v>Sick</v>
@@ -685,12 +685,104 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
+        <v>Sick (Dengu)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EMP009</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Akash</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Sick</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>EMP009</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Akash</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-07-30</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-07-30</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Sick</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -774,10 +866,10 @@
         <v>5</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -809,10 +901,10 @@
         <v>5</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1054,10 +1146,10 @@
         <v>5</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I10">
         <v>0</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-14T05:45:45.847Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,16 +621,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B2" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E2" t="str">
         <v>Sick</v>
@@ -639,15 +639,15 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>Sick</v>
+        <v>Sick Dengu</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B3" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C3" t="str">
         <v>2026-08-12</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B4" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C4" t="str">
         <v>2026-08-12</v>
@@ -685,7 +685,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="5">
@@ -696,10 +696,10 @@
         <v>Akash</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E5" t="str">
         <v>Sick</v>
@@ -708,67 +708,67 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>Sick</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B6" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E6" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B7" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-07-16</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-07-16</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E7" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP008</v>
+        <v>EMP009</v>
       </c>
       <c r="B8" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Akash</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E8" t="str">
         <v>Sick</v>
@@ -780,9 +780,55 @@
         <v>Sick</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Sick</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1067,10 +1113,10 @@
         <v>12</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F8">
         <v>5</v>
@@ -1146,10 +1192,10 @@
         <v>5</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10">
         <v>0</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-14T05:46:50.505Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,16 +621,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP009</v>
+        <v>EMP011</v>
       </c>
       <c r="B2" t="str">
-        <v>Akash</v>
+        <v>Dipaknath Jogi</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E2" t="str">
         <v>Sick</v>
@@ -639,21 +639,21 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>Sick Dengu</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B3" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E3" t="str">
         <v>Sick</v>
@@ -662,15 +662,15 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>Sick</v>
+        <v>Sick Dengu</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B4" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C4" t="str">
         <v>2026-08-12</v>
@@ -690,10 +690,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B5" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C5" t="str">
         <v>2026-08-12</v>
@@ -708,53 +708,53 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B6" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C6" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E6" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B7" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E7" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="8">
@@ -765,10 +765,10 @@
         <v>Akash</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E8" t="str">
         <v>Sick</v>
@@ -782,53 +782,76 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B9" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E9" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>EMP008</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>Vinod Vishwakarma</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C11" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D11" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="E10" t="str">
+      <c r="E11" t="str">
         <v>Sick</v>
       </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10" t="str">
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1262,10 +1285,10 @@
         <v>5</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I12">
         <v>0</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-21T13:57:14.930Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -667,33 +667,33 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP002</v>
+        <v>EMP007</v>
       </c>
       <c r="B4" t="str">
-        <v>Arvind</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E4" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B5" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C5" t="str">
         <v>2026-08-12</v>
@@ -713,10 +713,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B6" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C6" t="str">
         <v>2026-08-12</v>
@@ -731,53 +731,53 @@
         <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B7" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C7" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E7" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B8" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E8" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="9">
@@ -788,10 +788,10 @@
         <v>Akash</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E9" t="str">
         <v>Sick</v>
@@ -805,53 +805,76 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B10" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E10" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>EMP008</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>Vinod Vishwakarma</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C12" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D12" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E12" t="str">
         <v>Sick</v>
       </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="str">
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1136,10 +1159,10 @@
         <v>12</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F8">
         <v>5</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-21T14:14:27.648Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -690,22 +690,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B5" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-15</v>
       </c>
       <c r="E5" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5" t="str">
         <v>Sick</v>
@@ -713,10 +713,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B6" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C6" t="str">
         <v>2026-08-12</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B7" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C7" t="str">
         <v>2026-08-12</v>
@@ -754,53 +754,53 @@
         <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B8" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C8" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E8" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B9" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E9" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="10">
@@ -811,10 +811,10 @@
         <v>Akash</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E10" t="str">
         <v>Sick</v>
@@ -828,53 +828,76 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B11" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D11" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E11" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>EMP008</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B13" t="str">
         <v>Vinod Vishwakarma</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C13" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D13" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="E12" t="str">
+      <c r="E13" t="str">
         <v>Sick</v>
       </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12" t="str">
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1229,10 +1252,10 @@
         <v>12</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F10">
         <v>5</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-21T14:15:32.795Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,16 +621,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP011</v>
+        <v>EMP009</v>
       </c>
       <c r="B2" t="str">
-        <v>Dipaknath Jogi</v>
+        <v>Akash</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="E2" t="str">
         <v>Sick</v>
@@ -639,21 +639,21 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP009</v>
+        <v>EMP011</v>
       </c>
       <c r="B3" t="str">
-        <v>Akash</v>
+        <v>Dipaknath Jogi</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E3" t="str">
         <v>Sick</v>
@@ -662,84 +662,84 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>Sick Dengu</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B4" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C4" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E4" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick Dengu</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B5" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C5" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-08-15</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E5" t="str">
         <v>Earned</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B6" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-15</v>
       </c>
       <c r="E6" t="str">
         <v>Sick</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6" t="str">
-        <v>Sick</v>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B7" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C7" t="str">
         <v>2026-08-12</v>
@@ -759,10 +759,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B8" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C8" t="str">
         <v>2026-08-12</v>
@@ -777,53 +777,53 @@
         <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B9" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C9" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E9" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B10" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E10" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="11">
@@ -834,10 +834,10 @@
         <v>Akash</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D11" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E11" t="str">
         <v>Sick</v>
@@ -851,53 +851,76 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B12" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E12" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EMP008</v>
+        <v>EMP002</v>
       </c>
       <c r="B13" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Arvind</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="D13" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="E13" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1252,19 +1275,19 @@
         <v>12</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F10">
         <v>5</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="I10">
         <v>0</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-22T05:37:51.642Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,39 +621,39 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP009</v>
+        <v>EMP008</v>
       </c>
       <c r="B2" t="str">
-        <v>Akash</v>
+        <v>Vinod Vishwakarma</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-20</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-21</v>
       </c>
       <c r="E2" t="str">
         <v>Sick</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" t="str">
-        <v>Dengu</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP011</v>
+        <v>EMP009</v>
       </c>
       <c r="B3" t="str">
-        <v>Dipaknath Jogi</v>
+        <v>Akash</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="E3" t="str">
         <v>Sick</v>
@@ -662,21 +662,21 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP009</v>
+        <v>EMP011</v>
       </c>
       <c r="B4" t="str">
-        <v>Akash</v>
+        <v>Dipaknath Jogi</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E4" t="str">
         <v>Sick</v>
@@ -685,84 +685,84 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>Sick Dengu</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B5" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C5" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E5" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick Dengu</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B6" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C6" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-08-15</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E6" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" t="str">
-        <v>Dengu</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B7" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-15</v>
       </c>
       <c r="E7" t="str">
         <v>Sick</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7" t="str">
-        <v>Sick</v>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B8" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C8" t="str">
         <v>2026-08-12</v>
@@ -782,10 +782,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B9" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C9" t="str">
         <v>2026-08-12</v>
@@ -800,53 +800,53 @@
         <v>1</v>
       </c>
       <c r="G9" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B10" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C10" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E10" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B11" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D11" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E11" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="12">
@@ -857,10 +857,10 @@
         <v>Akash</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E12" t="str">
         <v>Sick</v>
@@ -874,53 +874,76 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B13" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D13" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E13" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>EMP008</v>
+        <v>EMP002</v>
       </c>
       <c r="B14" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Arvind</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="D14" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="E14" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1249,10 +1272,10 @@
         <v>5</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I9">
         <v>0</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-22T05:38:23.475Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,62 +621,62 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP008</v>
+        <v>EMP002</v>
       </c>
       <c r="B2" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Arvind</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08-20</v>
+        <v>2026-08-22</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-22</v>
       </c>
       <c r="E2" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>Sick</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP009</v>
+        <v>EMP008</v>
       </c>
       <c r="B3" t="str">
-        <v>Akash</v>
+        <v>Vinod Vishwakarma</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-20</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-21</v>
       </c>
       <c r="E3" t="str">
         <v>Sick</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" t="str">
-        <v>Dengu</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP011</v>
+        <v>EMP009</v>
       </c>
       <c r="B4" t="str">
-        <v>Dipaknath Jogi</v>
+        <v>Akash</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="E4" t="str">
         <v>Sick</v>
@@ -685,21 +685,21 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP009</v>
+        <v>EMP011</v>
       </c>
       <c r="B5" t="str">
-        <v>Akash</v>
+        <v>Dipaknath Jogi</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E5" t="str">
         <v>Sick</v>
@@ -708,84 +708,84 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>Sick Dengu</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B6" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C6" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E6" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick Dengu</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B7" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C7" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-08-15</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E7" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G7" t="str">
-        <v>Dengu</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B8" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-15</v>
       </c>
       <c r="E8" t="str">
         <v>Sick</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G8" t="str">
-        <v>Sick</v>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B9" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C9" t="str">
         <v>2026-08-12</v>
@@ -805,10 +805,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B10" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C10" t="str">
         <v>2026-08-12</v>
@@ -823,53 +823,53 @@
         <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B11" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C11" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D11" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E11" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B12" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E12" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="13">
@@ -880,10 +880,10 @@
         <v>Akash</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D13" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E13" t="str">
         <v>Sick</v>
@@ -897,53 +897,76 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B14" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D14" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E14" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>EMP008</v>
+        <v>EMP002</v>
       </c>
       <c r="B15" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Arvind</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="D15" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="E15" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>EMP008</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Vinod Vishwakarma</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1053,10 +1076,10 @@
         <v>12</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3">
         <v>5</v>

</xml_diff>

<commit_message>
Update leave data - 2026-08-22T05:39:57.282Z
</commit_message>
<xml_diff>
--- a/data/leave-data.xlsx
+++ b/data/leave-data.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -644,62 +644,62 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP008</v>
+        <v>EMP011</v>
       </c>
       <c r="B3" t="str">
-        <v>Vinod Vishwakarma</v>
+        <v>Dipaknath Jogi</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-08-20</v>
+        <v>2026-08-22</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-22</v>
       </c>
       <c r="E3" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>Sick</v>
+        <v>Went Village</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP009</v>
+        <v>EMP008</v>
       </c>
       <c r="B4" t="str">
-        <v>Akash</v>
+        <v>Vinod Vishwakarma</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-20</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-21</v>
       </c>
       <c r="E4" t="str">
         <v>Sick</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="str">
-        <v>Dengu</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EMP011</v>
+        <v>EMP009</v>
       </c>
       <c r="B5" t="str">
-        <v>Dipaknath Jogi</v>
+        <v>Akash</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-17</v>
       </c>
       <c r="E5" t="str">
         <v>Sick</v>
@@ -708,21 +708,21 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EMP009</v>
+        <v>EMP011</v>
       </c>
       <c r="B6" t="str">
-        <v>Akash</v>
+        <v>Dipaknath Jogi</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E6" t="str">
         <v>Sick</v>
@@ -731,84 +731,84 @@
         <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>Sick Dengu</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B7" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C7" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-08-14</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E7" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick Dengu</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B8" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C8" t="str">
         <v>2026-08-13</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-08-15</v>
+        <v>2026-08-14</v>
       </c>
       <c r="E8" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="str">
-        <v>Dengu</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B9" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-13</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-15</v>
       </c>
       <c r="E9" t="str">
         <v>Sick</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G9" t="str">
-        <v>Sick</v>
+        <v>Dengu</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EMP001</v>
+        <v>EMP002</v>
       </c>
       <c r="B10" t="str">
-        <v>Anil Kumar Sharma</v>
+        <v>Arvind</v>
       </c>
       <c r="C10" t="str">
         <v>2026-08-12</v>
@@ -828,10 +828,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EMP009</v>
+        <v>EMP001</v>
       </c>
       <c r="B11" t="str">
-        <v>Akash</v>
+        <v>Anil Kumar Sharma</v>
       </c>
       <c r="C11" t="str">
         <v>2026-08-12</v>
@@ -846,53 +846,53 @@
         <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v>Sick (Dengu)</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>EMP007</v>
+        <v>EMP009</v>
       </c>
       <c r="B12" t="str">
-        <v>Vikash Sharma</v>
+        <v>Akash</v>
       </c>
       <c r="C12" t="str">
         <v>2026-08-12</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-08-13</v>
+        <v>2026-08-12</v>
       </c>
       <c r="E12" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v>Take care of Akash in Hospital</v>
+        <v>Sick (Dengu)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EMP009</v>
+        <v>EMP007</v>
       </c>
       <c r="B13" t="str">
-        <v>Akash</v>
+        <v>Vikash Sharma</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
       <c r="D13" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-13</v>
       </c>
       <c r="E13" t="str">
-        <v>Sick</v>
+        <v>Earned</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" t="str">
-        <v>Sick</v>
+        <v>Take care of Akash in Hospital</v>
       </c>
     </row>
     <row r="14">
@@ -903,10 +903,10 @@
         <v>Akash</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="D14" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E14" t="str">
         <v>Sick</v>
@@ -920,53 +920,76 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>EMP002</v>
+        <v>EMP009</v>
       </c>
       <c r="B15" t="str">
-        <v>Arvind</v>
+        <v>Akash</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="D15" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
       <c r="E15" t="str">
-        <v>Earned</v>
+        <v>Sick</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>jagannath Ratra</v>
+        <v>Sick</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>EMP002</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Arvind</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Earned</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" t="str">
+        <v>jagannath Ratra</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>EMP008</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B17" t="str">
         <v>Vinod Vishwakarma</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C17" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D17" t="str">
         <v>2026-07-14</v>
       </c>
-      <c r="E16" t="str">
-        <v>Sick</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-      <c r="G16" t="str">
+      <c r="E17" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" t="str">
         <v>Sick</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1391,10 +1414,10 @@
         <v>12</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F12">
         <v>5</v>

</xml_diff>